<commit_message>
added progress status + improved references
</commit_message>
<xml_diff>
--- a/Map/USDM2FHIR.xlsx
+++ b/Map/USDM2FHIR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_db\Map\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25BDAC8F-9522-4D82-8D00-852D587BA91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B883B70-A178-4D5A-A7DB-BFB29AD83B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9045" yWindow="-19740" windowWidth="22320" windowHeight="17160" xr2:uid="{97BCDFE6-590C-45E1-8F75-1AA7EE2945FF}"/>
+    <workbookView xWindow="-9090" yWindow="-14685" windowWidth="31170" windowHeight="13635" xr2:uid="{97BCDFE6-590C-45E1-8F75-1AA7EE2945FF}"/>
   </bookViews>
   <sheets>
     <sheet name="USDM2FHIR map" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="285">
   <si>
     <t>Item</t>
   </si>
@@ -896,9 +896,6 @@
     <t>study.versions.organizations.managedSites.{id: id}</t>
   </si>
   <si>
-    <t>site.reference</t>
-  </si>
-  <si>
     <t>location reference</t>
   </si>
   <si>
@@ -983,12 +980,6 @@
     <t>purposeType.coding</t>
   </si>
   <si>
-    <t>study.versions.studyDesigns.objectives@$ob.$ob.endpoints.(
-    $firstWord := function($s) {$split($s, " ")[0]};
-    $titleCase := function($s) {$join($split($lowercase($s), " ")@$w.($uppercase($substring($w, 0, 1)) &amp; $substring($w, 1))," ")};
-{$ob.id: {"code:":$lowercase($firstWord(level.decode)), "display": $titleCase($firstWord(level.decode)), "system": "http://terminology.hl7.org/CodeSystem/research-study-objective-type"}})</t>
-  </si>
-  <si>
     <t>Endpoint level</t>
   </si>
   <si>
@@ -1043,13 +1034,71 @@
   </si>
   <si>
     <t>purpose _ intent</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives@$ob.$ob.endpoints.(
+    $firstWord := function($s) {$split($s, " ")[0]};
+    $titleCase := function($s) {$join($split($lowercase($s), " ")@$w.($uppercase($substring($w, 0, 1)) &amp; $substring($w, 1))," ")};
+{$ob.id: {"code":$lowercase($firstWord(level.decode)), "display": $titleCase($firstWord(level.decode)), "system": "http://terminology.hl7.org/CodeSystem/research-study-objective-type"}})</t>
+  </si>
+  <si>
+    <t>progress status</t>
+  </si>
+  <si>
+    <t>progressStatus.state.coding</t>
+  </si>
+  <si>
+    <t>progressStatus</t>
+  </si>
+  <si>
+    <t>extension studyProgressStatus</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>progress status actual</t>
+  </si>
+  <si>
+    <t>progressStatus.actual</t>
+  </si>
+  <si>
+    <t>isActual</t>
+  </si>
+  <si>
+    <t>progress status period</t>
+  </si>
+  <si>
+    <t>(study.versions.extensionAttributes.extensionAttributes.valueExtensionClass[url="https://cdisc.org/usdm/extension-studyProgressStatus/class1"])@$rp.$rp.extensionAttributes[url="https://cdisc.org/usdm/extension-studyProgressStatus-1/attribute-state"].
+{$rp.id:{"code": valueCode.code, "display": valueCode.decode, "system": valueCode.codeSystem}}</t>
+  </si>
+  <si>
+    <t>(study.versions.extensionAttributes.extensionAttributes.valueExtensionClass[url="https://cdisc.org/usdm/extension-studyProgressStatus/class1"])@$rp.$rp.extensionAttributes[url="https://cdisc.org/usdm/extension-studyProgressStatus-1/attribute-isActive"].
+{$rp.id:valueBoolean}</t>
+  </si>
+  <si>
+    <t>(study.versions.extensionAttributes.extensionAttributes.valueExtensionClass[url="https://cdisc.org/usdm/extension-studyProgressStatus/class1"])@$rp.
+{$rp.id: {"start" : $rp.extensionAttributes[url="https://cdisc.org/usdm/extension-studyProgressStatus-1/attribute-startDate"].valueString,
+            "end" : $rp.extensionAttributes[url="https://cdisc.org/usdm/extension-studyProgressStatus-1/attribute-endDate"].valueString}}</t>
+  </si>
+  <si>
+    <t>progressStatus.period</t>
+  </si>
+  <si>
+    <t>startDate, endDate</t>
+  </si>
+  <si>
+    <t>{"eligibility-criteria": {"reference": "eligibility-criteria", "type":"Group"}}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">study.versions.organizations.managedSites.{id: {"reference": id, "type":"Location"}} </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1079,6 +1128,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1100,7 +1157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1116,6 +1173,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1453,7 +1511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81DD2990-A668-4ED7-89E0-40F5440ED267}">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.1796875" style="3" customWidth="1"/>
@@ -1516,13 +1574,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C3" t="s">
         <v>181</v>
       </c>
       <c r="D3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
@@ -1539,7 +1597,7 @@
         <v>82</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C4" t="s">
         <v>181</v>
@@ -1562,7 +1620,7 @@
         <v>83</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C5" t="s">
         <v>181</v>
@@ -1599,10 +1657,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C7" t="s">
         <v>181</v>
@@ -1662,16 +1720,16 @@
     </row>
     <row r="10" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C10" t="s">
         <v>181</v>
       </c>
       <c r="D10" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E10" t="s">
         <v>9</v>
@@ -1685,10 +1743,10 @@
     </row>
     <row r="11" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C11" t="s">
         <v>181</v>
@@ -1703,21 +1761,21 @@
         <v>136</v>
       </c>
       <c r="G11" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C12" t="s">
         <v>181</v>
       </c>
       <c r="D12" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E12" t="s">
         <v>9</v>
@@ -1731,16 +1789,16 @@
     </row>
     <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C13" t="s">
         <v>181</v>
       </c>
       <c r="D13" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="E13" t="s">
         <v>9</v>
@@ -1749,7 +1807,7 @@
         <v>136</v>
       </c>
       <c r="G13" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -2001,16 +2059,16 @@
     </row>
     <row r="25" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
       <c r="C25" t="s">
         <v>181</v>
       </c>
       <c r="D25" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E25" t="s">
         <v>60</v>
@@ -2024,16 +2082,16 @@
     </row>
     <row r="26" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C26" t="s">
         <v>181</v>
       </c>
       <c r="D26" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E26" t="s">
         <v>107</v>
@@ -2041,16 +2099,16 @@
     </row>
     <row r="27" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>249</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>250</v>
       </c>
       <c r="C27" t="s">
         <v>181</v>
       </c>
       <c r="D27" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E27" t="s">
         <v>77</v>
@@ -2062,178 +2120,178 @@
         <v>144</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>234</v>
+        <v>269</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>232</v>
+        <v>278</v>
       </c>
       <c r="C28" t="s">
         <v>181</v>
       </c>
       <c r="D28" t="s">
-        <v>233</v>
+        <v>270</v>
       </c>
       <c r="E28" t="s">
-        <v>90</v>
-      </c>
-      <c r="F28" t="s">
-        <v>145</v>
-      </c>
-      <c r="G28" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+        <v>271</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>235</v>
+        <v>274</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>232</v>
+        <v>279</v>
       </c>
       <c r="C29" t="s">
-        <v>236</v>
+        <v>181</v>
       </c>
       <c r="D29" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+        <v>275</v>
+      </c>
+      <c r="E29" t="s">
+        <v>271</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>89</v>
+        <v>277</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>88</v>
+        <v>280</v>
       </c>
       <c r="C30" t="s">
-        <v>236</v>
+        <v>181</v>
       </c>
       <c r="D30" t="s">
-        <v>237</v>
-      </c>
-      <c r="F30" t="s">
-        <v>145</v>
-      </c>
-      <c r="G30" t="s">
-        <v>9</v>
+        <v>281</v>
+      </c>
+      <c r="E30" t="s">
+        <v>271</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>91</v>
+        <v>233</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>92</v>
+        <v>284</v>
       </c>
       <c r="C31" t="s">
-        <v>236</v>
+        <v>181</v>
       </c>
       <c r="D31" t="s">
-        <v>137</v>
+        <v>90</v>
+      </c>
+      <c r="E31" t="s">
+        <v>90</v>
+      </c>
+      <c r="F31" t="s">
+        <v>145</v>
+      </c>
+      <c r="G31" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
-        <v>94</v>
+        <v>234</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>93</v>
+        <v>232</v>
       </c>
       <c r="C32" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D32" t="s">
-        <v>238</v>
-      </c>
-      <c r="F32" t="s">
-        <v>145</v>
-      </c>
-      <c r="G32" t="s">
-        <v>146</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
-        <v>181</v>
+        <v>235</v>
       </c>
       <c r="D33" t="s">
-        <v>103</v>
-      </c>
-      <c r="E33" t="s">
-        <v>19</v>
+        <v>236</v>
       </c>
       <c r="F33" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G33" t="s">
-        <v>148</v>
+        <v>9</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="3" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C34" t="s">
-        <v>181</v>
+        <v>235</v>
       </c>
       <c r="D34" t="s">
-        <v>104</v>
-      </c>
-      <c r="E34" t="s">
-        <v>19</v>
-      </c>
-      <c r="F34" t="s">
-        <v>147</v>
-      </c>
-      <c r="G34" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="3" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C35" t="s">
-        <v>181</v>
+        <v>235</v>
       </c>
       <c r="D35" t="s">
-        <v>103</v>
-      </c>
-      <c r="E35" t="s">
-        <v>19</v>
+        <v>237</v>
       </c>
       <c r="F35" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G35" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C36" t="s">
         <v>181</v>
       </c>
       <c r="D36" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E36" t="s">
         <v>19</v>
@@ -2245,277 +2303,277 @@
         <v>148</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="3" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="C37" t="s">
         <v>181</v>
       </c>
       <c r="D37" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E37" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="F37" t="s">
+        <v>147</v>
+      </c>
+      <c r="G37" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="3" t="s">
-        <v>230</v>
+        <v>99</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>183</v>
+        <v>101</v>
       </c>
       <c r="C38" t="s">
         <v>181</v>
       </c>
       <c r="D38" t="s">
-        <v>229</v>
+        <v>103</v>
       </c>
       <c r="E38" t="s">
-        <v>231</v>
+        <v>19</v>
+      </c>
+      <c r="F38" t="s">
+        <v>147</v>
+      </c>
+      <c r="G38" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C39" t="s">
+        <v>181</v>
+      </c>
+      <c r="D39" t="s">
+        <v>104</v>
+      </c>
+      <c r="E39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F39" t="s">
+        <v>147</v>
+      </c>
+      <c r="G39" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A40" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C40" t="s">
+        <v>181</v>
+      </c>
+      <c r="D40" t="s">
+        <v>108</v>
+      </c>
+      <c r="E40" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A41" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="C41" t="s">
+        <v>181</v>
+      </c>
+      <c r="D41" t="s">
+        <v>229</v>
+      </c>
+      <c r="E41" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B42" s="3" t="s">
         <v>183</v>
-      </c>
-      <c r="C39" t="s">
-        <v>187</v>
-      </c>
-      <c r="D39" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A40" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C40" t="s">
-        <v>187</v>
-      </c>
-      <c r="D40" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A41" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="C41" t="s">
-        <v>187</v>
-      </c>
-      <c r="D41" t="s">
-        <v>185</v>
-      </c>
-      <c r="E41" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A42" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>188</v>
       </c>
       <c r="C42" t="s">
         <v>187</v>
       </c>
       <c r="D42" t="s">
-        <v>152</v>
-      </c>
-      <c r="E42" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C43" t="s">
         <v>187</v>
       </c>
       <c r="D43" t="s">
-        <v>35</v>
-      </c>
-      <c r="E43" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>36</v>
+        <v>184</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="C44" t="s">
         <v>187</v>
       </c>
       <c r="D44" t="s">
-        <v>37</v>
+        <v>185</v>
       </c>
       <c r="E44" t="s">
         <v>172</v>
       </c>
-      <c r="F44" t="s">
-        <v>149</v>
-      </c>
-      <c r="G44" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+    </row>
+    <row r="45" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>197</v>
+        <v>169</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C45" t="s">
-        <v>21</v>
+        <v>187</v>
       </c>
       <c r="D45" t="s">
-        <v>38</v>
-      </c>
-      <c r="F45" t="s">
-        <v>149</v>
-      </c>
-      <c r="G45" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+        <v>152</v>
+      </c>
+      <c r="E45" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C46" t="s">
-        <v>21</v>
+        <v>187</v>
       </c>
       <c r="D46" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+      <c r="E46" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>200</v>
+        <v>36</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="C47" t="s">
-        <v>21</v>
+        <v>187</v>
       </c>
       <c r="D47" t="s">
-        <v>22</v>
+        <v>37</v>
+      </c>
+      <c r="E47" t="s">
+        <v>172</v>
       </c>
       <c r="F47" t="s">
         <v>149</v>
       </c>
       <c r="G47" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="116" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="C48" t="s">
         <v>21</v>
       </c>
       <c r="D48" t="s">
-        <v>23</v>
-      </c>
-      <c r="E48" t="s">
-        <v>172</v>
+        <v>38</v>
       </c>
       <c r="F48" t="s">
         <v>149</v>
       </c>
       <c r="G48" t="s">
-        <v>150</v>
+        <v>38</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="C49" t="s">
         <v>21</v>
       </c>
       <c r="D49" t="s">
-        <v>24</v>
-      </c>
-      <c r="E49" t="s">
-        <v>172</v>
-      </c>
-      <c r="F49" t="s">
-        <v>149</v>
-      </c>
-      <c r="G49" t="s">
-        <v>150</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="C50" t="s">
         <v>21</v>
       </c>
       <c r="D50" t="s">
-        <v>25</v>
-      </c>
-      <c r="E50" t="s">
-        <v>172</v>
+        <v>22</v>
       </c>
       <c r="F50" t="s">
         <v>149</v>
       </c>
       <c r="G50" t="s">
-        <v>150</v>
+        <v>9</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="C51" t="s">
         <v>21</v>
       </c>
       <c r="D51" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E51" t="s">
         <v>172</v>
@@ -2529,16 +2587,16 @@
     </row>
     <row r="52" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="C52" t="s">
         <v>21</v>
       </c>
       <c r="D52" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E52" t="s">
         <v>172</v>
@@ -2547,21 +2605,21 @@
         <v>149</v>
       </c>
       <c r="G52" t="s">
-        <v>22</v>
+        <v>150</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>241</v>
+        <v>211</v>
       </c>
       <c r="C53" t="s">
         <v>21</v>
       </c>
       <c r="D53" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="E53" t="s">
         <v>172</v>
@@ -2570,21 +2628,21 @@
         <v>149</v>
       </c>
       <c r="G53" t="s">
-        <v>132</v>
+        <v>150</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="C54" t="s">
         <v>21</v>
       </c>
       <c r="D54" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E54" t="s">
         <v>172</v>
@@ -2593,21 +2651,21 @@
         <v>149</v>
       </c>
       <c r="G54" t="s">
-        <v>132</v>
+        <v>150</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>206</v>
+        <v>220</v>
       </c>
       <c r="C55" t="s">
         <v>21</v>
       </c>
       <c r="D55" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E55" t="s">
         <v>172</v>
@@ -2616,21 +2674,21 @@
         <v>149</v>
       </c>
       <c r="G55" t="s">
-        <v>132</v>
+        <v>22</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>193</v>
+        <v>202</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>221</v>
+        <v>240</v>
       </c>
       <c r="C56" t="s">
         <v>21</v>
       </c>
       <c r="D56" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E56" t="s">
         <v>172</v>
@@ -2639,21 +2697,21 @@
         <v>149</v>
       </c>
       <c r="G56" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>31</v>
+        <v>203</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>222</v>
+        <v>205</v>
       </c>
       <c r="C57" t="s">
         <v>21</v>
       </c>
       <c r="D57" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E57" t="s">
         <v>172</v>
@@ -2662,21 +2720,21 @@
         <v>149</v>
       </c>
       <c r="G57" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>110</v>
+        <v>204</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>223</v>
+        <v>206</v>
       </c>
       <c r="C58" t="s">
         <v>21</v>
       </c>
       <c r="D58" t="s">
-        <v>111</v>
+        <v>30</v>
       </c>
       <c r="E58" t="s">
         <v>172</v>
@@ -2685,21 +2743,21 @@
         <v>149</v>
       </c>
       <c r="G58" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>116</v>
+        <v>193</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C59" t="s">
         <v>21</v>
       </c>
       <c r="D59" t="s">
-        <v>120</v>
+        <v>32</v>
       </c>
       <c r="E59" t="s">
         <v>172</v>
@@ -2708,21 +2766,21 @@
         <v>149</v>
       </c>
       <c r="G59" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>112</v>
+        <v>31</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C60" t="s">
         <v>21</v>
       </c>
       <c r="D60" t="s">
-        <v>113</v>
+        <v>33</v>
       </c>
       <c r="E60" t="s">
         <v>172</v>
@@ -2731,21 +2789,21 @@
         <v>149</v>
       </c>
       <c r="G60" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C61" t="s">
         <v>21</v>
       </c>
       <c r="D61" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="E61" t="s">
         <v>172</v>
@@ -2759,110 +2817,180 @@
     </row>
     <row r="62" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C62" t="s">
         <v>21</v>
       </c>
       <c r="D62" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E62" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="63" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="F62" t="s">
+        <v>149</v>
+      </c>
+      <c r="G62" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C63" t="s">
         <v>21</v>
       </c>
       <c r="D63" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="E63" t="s">
         <v>172</v>
       </c>
+      <c r="F63" t="s">
+        <v>149</v>
+      </c>
+      <c r="G63" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="64" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C64" t="s">
         <v>21</v>
       </c>
       <c r="D64" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="E64" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+      <c r="F64" t="s">
+        <v>149</v>
+      </c>
+      <c r="G64" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>242</v>
+        <v>121</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>243</v>
+        <v>226</v>
       </c>
       <c r="C65" t="s">
         <v>21</v>
       </c>
       <c r="D65" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
       <c r="E65" t="s">
         <v>172</v>
       </c>
-      <c r="F65" t="s">
-        <v>153</v>
-      </c>
-      <c r="G65" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" ht="203" x14ac:dyDescent="0.35">
+    </row>
+    <row r="66" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
-        <v>170</v>
+        <v>125</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="C66" t="s">
         <v>21</v>
       </c>
       <c r="D66" t="s">
-        <v>240</v>
+        <v>123</v>
       </c>
       <c r="E66" t="s">
         <v>172</v>
       </c>
-      <c r="F66" t="s">
+    </row>
+    <row r="67" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A67" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C67" t="s">
+        <v>21</v>
+      </c>
+      <c r="D67" t="s">
+        <v>124</v>
+      </c>
+      <c r="E67" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+      <c r="A68" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="C68" t="s">
+        <v>21</v>
+      </c>
+      <c r="D68" t="s">
+        <v>152</v>
+      </c>
+      <c r="E68" t="s">
+        <v>172</v>
+      </c>
+      <c r="F68" t="s">
+        <v>153</v>
+      </c>
+      <c r="G68" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="203" x14ac:dyDescent="0.35">
+      <c r="A69" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="C69" t="s">
+        <v>21</v>
+      </c>
+      <c r="D69" t="s">
+        <v>239</v>
+      </c>
+      <c r="E69" t="s">
+        <v>172</v>
+      </c>
+      <c r="F69" t="s">
         <v>171</v>
       </c>
-      <c r="G66" t="s">
+      <c r="G69" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B67" s="3"/>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B68" s="3"/>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B70" s="3"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="B71" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B25" r:id="rId1" display="study.versions.studyDesigns.objectives@$ob.$ob.endpoints[level.code=&quot;C94496&quot;].{$ob.id: &quot;primary&quot;}" xr:uid="{74E81704-A140-48FF-9D58-8B18F3C8EA13}"/>
+    <hyperlink ref="B11" r:id="rId2" xr:uid="{546F8543-000B-4AD4-8472-81E6831062E9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2888,10 +3016,10 @@
       </c>
     </row>
     <row r="3" spans="1:2" s="3" customFormat="1" ht="45.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="B3" s="7"/>
+      <c r="B3" s="8"/>
     </row>
     <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
@@ -3127,6 +3255,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4">
@@ -3137,7 +3274,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100527ED9A1E2F34D48AA5925CCBA0CEC41" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="73c2da0cd5c8d9fd369ff3018c825410">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4" xmlns:ns3="985d26ac-cf7b-4687-94e0-26b141782da7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b3600b0f37fd05e6cabe55b41d10e7dc" ns2:_="" ns3:_="">
     <xsd:import namespace="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4"/>
@@ -3332,16 +3469,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12DB76A7-ED98-4EE3-9432-17F601352CF4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E61FE636-68A4-4725-8134-F4B9672BB2E7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -3358,7 +3494,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9675DCA-D684-4E4E-B61D-0AB2D6821582}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3375,12 +3511,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12DB76A7-ED98-4EE3-9432-17F601352CF4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
resolved some small bugs
</commit_message>
<xml_diff>
--- a/Map/USDM2FHIR.xlsx
+++ b/Map/USDM2FHIR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_db\Map\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B883B70-A178-4D5A-A7DB-BFB29AD83B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8114FA2F-D3DF-4F6E-960A-13CB9A583246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-9090" yWindow="-14685" windowWidth="31170" windowHeight="13635" xr2:uid="{97BCDFE6-590C-45E1-8F75-1AA7EE2945FF}"/>
+    <workbookView xWindow="8685" yWindow="-18390" windowWidth="22320" windowHeight="16680" xr2:uid="{97BCDFE6-590C-45E1-8F75-1AA7EE2945FF}"/>
   </bookViews>
   <sheets>
     <sheet name="USDM2FHIR map" sheetId="1" r:id="rId1"/>
@@ -958,9 +958,6 @@
     <t>study.versions.studyIdentifiers.{id: text}</t>
   </si>
   <si>
-    <t>(study.versions)@$sv.$sv.studyIdentifiers@$id.{id: $sv.organizations[id=$id.scopeId].label}</t>
-  </si>
-  <si>
     <t>phase.coding</t>
   </si>
   <si>
@@ -1092,6 +1089,9 @@
   </si>
   <si>
     <t xml:space="preserve">study.versions.organizations.managedSites.{id: {"reference": id, "type":"Location"}} </t>
+  </si>
+  <si>
+    <t>(study.versions)@$sv.$sv.studyIdentifiers@$id.$id{id: $sv.organizations[id=$id.scopeId].label}</t>
   </si>
 </sst>
 </file>
@@ -1574,13 +1574,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C3" t="s">
         <v>181</v>
       </c>
       <c r="D3" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
@@ -1620,7 +1620,7 @@
         <v>83</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>246</v>
+        <v>284</v>
       </c>
       <c r="C5" t="s">
         <v>181</v>
@@ -1720,16 +1720,16 @@
     </row>
     <row r="10" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>254</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>255</v>
       </c>
       <c r="C10" t="s">
         <v>181</v>
       </c>
       <c r="D10" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E10" t="s">
         <v>9</v>
@@ -1743,10 +1743,10 @@
     </row>
     <row r="11" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>259</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>260</v>
       </c>
       <c r="C11" t="s">
         <v>181</v>
@@ -1761,21 +1761,21 @@
         <v>136</v>
       </c>
       <c r="G11" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>262</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>263</v>
       </c>
       <c r="C12" t="s">
         <v>181</v>
       </c>
       <c r="D12" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E12" t="s">
         <v>9</v>
@@ -1789,16 +1789,16 @@
     </row>
     <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>264</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>265</v>
       </c>
       <c r="C13" t="s">
         <v>181</v>
       </c>
       <c r="D13" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E13" t="s">
         <v>9</v>
@@ -1807,7 +1807,7 @@
         <v>136</v>
       </c>
       <c r="G13" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -2059,16 +2059,16 @@
     </row>
     <row r="25" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C25" t="s">
         <v>181</v>
       </c>
       <c r="D25" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E25" t="s">
         <v>60</v>
@@ -2082,16 +2082,16 @@
     </row>
     <row r="26" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C26" t="s">
         <v>181</v>
       </c>
       <c r="D26" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E26" t="s">
         <v>107</v>
@@ -2099,16 +2099,16 @@
     </row>
     <row r="27" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>248</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>249</v>
       </c>
       <c r="C27" t="s">
         <v>181</v>
       </c>
       <c r="D27" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E27" t="s">
         <v>77</v>
@@ -2122,71 +2122,71 @@
     </row>
     <row r="28" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C28" t="s">
         <v>181</v>
       </c>
       <c r="D28" t="s">
+        <v>269</v>
+      </c>
+      <c r="E28" t="s">
         <v>270</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="G28" s="7" t="s">
         <v>272</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C29" t="s">
         <v>181</v>
       </c>
       <c r="D29" t="s">
+        <v>274</v>
+      </c>
+      <c r="E29" t="s">
+        <v>270</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="G29" s="7" t="s">
         <v>275</v>
-      </c>
-      <c r="E29" t="s">
-        <v>271</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C30" t="s">
         <v>181</v>
       </c>
       <c r="D30" t="s">
+        <v>280</v>
+      </c>
+      <c r="E30" t="s">
+        <v>270</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="G30" s="7" t="s">
         <v>281</v>
-      </c>
-      <c r="E30" t="s">
-        <v>271</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
@@ -2194,7 +2194,7 @@
         <v>233</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C31" t="s">
         <v>181</v>
@@ -2394,7 +2394,7 @@
         <v>230</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C41" t="s">
         <v>181</v>
@@ -3264,17 +3264,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="985d26ac-cf7b-4687-94e0-26b141782da7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100527ED9A1E2F34D48AA5925CCBA0CEC41" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="73c2da0cd5c8d9fd369ff3018c825410">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4" xmlns:ns3="985d26ac-cf7b-4687-94e0-26b141782da7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b3600b0f37fd05e6cabe55b41d10e7dc" ns2:_="" ns3:_="">
     <xsd:import namespace="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4"/>
@@ -3469,6 +3458,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="985d26ac-cf7b-4687-94e0-26b141782da7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12DB76A7-ED98-4EE3-9432-17F601352CF4}">
   <ds:schemaRefs>
@@ -3478,23 +3478,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E61FE636-68A4-4725-8134-F4B9672BB2E7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="985d26ac-cf7b-4687-94e0-26b141782da7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9675DCA-D684-4E4E-B61D-0AB2D6821582}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3511,4 +3494,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E61FE636-68A4-4725-8134-F4B9672BB2E7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="985d26ac-cf7b-4687-94e0-26b141782da7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update map criteria description
</commit_message>
<xml_diff>
--- a/Map/USDM2FHIR.xlsx
+++ b/Map/USDM2FHIR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_db\Map\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8114FA2F-D3DF-4F6E-960A-13CB9A583246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDE9255-A218-4184-A17D-0B729E65BE66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8685" yWindow="-18390" windowWidth="22320" windowHeight="16680" xr2:uid="{97BCDFE6-590C-45E1-8F75-1AA7EE2945FF}"/>
+    <workbookView xWindow="-11700" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{97BCDFE6-590C-45E1-8F75-1AA7EE2945FF}"/>
   </bookViews>
   <sheets>
     <sheet name="USDM2FHIR map" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="284">
   <si>
     <t>Item</t>
   </si>
@@ -596,9 +596,6 @@
   </si>
   <si>
     <t>Eligibility criteria text</t>
-  </si>
-  <si>
-    <t>characteristic.valueCodeableConcept</t>
   </si>
   <si>
     <t>study.versions@$sv.(
@@ -1574,13 +1571,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C3" t="s">
         <v>181</v>
       </c>
       <c r="D3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
@@ -1597,7 +1594,7 @@
         <v>82</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C4" t="s">
         <v>181</v>
@@ -1620,7 +1617,7 @@
         <v>83</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C5" t="s">
         <v>181</v>
@@ -1657,10 +1654,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C7" t="s">
         <v>181</v>
@@ -1720,16 +1717,16 @@
     </row>
     <row r="10" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>253</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>254</v>
       </c>
       <c r="C10" t="s">
         <v>181</v>
       </c>
       <c r="D10" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E10" t="s">
         <v>9</v>
@@ -1743,10 +1740,10 @@
     </row>
     <row r="11" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>258</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>259</v>
       </c>
       <c r="C11" t="s">
         <v>181</v>
@@ -1761,21 +1758,21 @@
         <v>136</v>
       </c>
       <c r="G11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>261</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>262</v>
       </c>
       <c r="C12" t="s">
         <v>181</v>
       </c>
       <c r="D12" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E12" t="s">
         <v>9</v>
@@ -1789,16 +1786,16 @@
     </row>
     <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>263</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>264</v>
       </c>
       <c r="C13" t="s">
         <v>181</v>
       </c>
       <c r="D13" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E13" t="s">
         <v>9</v>
@@ -1807,7 +1804,7 @@
         <v>136</v>
       </c>
       <c r="G13" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="58" x14ac:dyDescent="0.35">
@@ -2059,16 +2056,16 @@
     </row>
     <row r="25" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C25" t="s">
         <v>181</v>
       </c>
       <c r="D25" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="E25" t="s">
         <v>60</v>
@@ -2082,16 +2079,16 @@
     </row>
     <row r="26" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C26" t="s">
         <v>181</v>
       </c>
       <c r="D26" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E26" t="s">
         <v>107</v>
@@ -2099,16 +2096,16 @@
     </row>
     <row r="27" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>247</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>248</v>
       </c>
       <c r="C27" t="s">
         <v>181</v>
       </c>
       <c r="D27" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E27" t="s">
         <v>77</v>
@@ -2122,79 +2119,79 @@
     </row>
     <row r="28" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C28" t="s">
         <v>181</v>
       </c>
       <c r="D28" t="s">
+        <v>268</v>
+      </c>
+      <c r="E28" t="s">
         <v>269</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F28" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="G28" s="7" t="s">
         <v>271</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C29" t="s">
         <v>181</v>
       </c>
       <c r="D29" t="s">
+        <v>273</v>
+      </c>
+      <c r="E29" t="s">
+        <v>269</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="G29" s="7" t="s">
         <v>274</v>
-      </c>
-      <c r="E29" t="s">
-        <v>270</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C30" t="s">
         <v>181</v>
       </c>
       <c r="D30" t="s">
+        <v>279</v>
+      </c>
+      <c r="E30" t="s">
+        <v>269</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="G30" s="7" t="s">
         <v>280</v>
-      </c>
-      <c r="E30" t="s">
-        <v>270</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>271</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C31" t="s">
         <v>181</v>
@@ -2214,13 +2211,13 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="C32" t="s">
         <v>234</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="C32" t="s">
-        <v>235</v>
       </c>
       <c r="D32" t="s">
         <v>38</v>
@@ -2234,10 +2231,10 @@
         <v>88</v>
       </c>
       <c r="C33" t="s">
+        <v>234</v>
+      </c>
+      <c r="D33" t="s">
         <v>235</v>
-      </c>
-      <c r="D33" t="s">
-        <v>236</v>
       </c>
       <c r="F33" t="s">
         <v>145</v>
@@ -2254,7 +2251,7 @@
         <v>92</v>
       </c>
       <c r="C34" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D34" t="s">
         <v>137</v>
@@ -2268,10 +2265,10 @@
         <v>93</v>
       </c>
       <c r="C35" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D35" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F35" t="s">
         <v>145</v>
@@ -2391,19 +2388,19 @@
     </row>
     <row r="41" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C41" t="s">
         <v>181</v>
       </c>
       <c r="D41" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E41" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
@@ -2414,7 +2411,7 @@
         <v>183</v>
       </c>
       <c r="C42" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D42" t="s">
         <v>38</v>
@@ -2422,13 +2419,13 @@
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C43" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D43" t="s">
         <v>34</v>
@@ -2439,13 +2436,13 @@
         <v>184</v>
       </c>
       <c r="B44" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C44" t="s">
         <v>186</v>
       </c>
-      <c r="C44" t="s">
-        <v>187</v>
-      </c>
       <c r="D44" t="s">
-        <v>185</v>
+        <v>27</v>
       </c>
       <c r="E44" t="s">
         <v>172</v>
@@ -2456,10 +2453,10 @@
         <v>169</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C45" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D45" t="s">
         <v>152</v>
@@ -2470,13 +2467,13 @@
     </row>
     <row r="46" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C46" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D46" t="s">
         <v>35</v>
@@ -2490,10 +2487,10 @@
         <v>36</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C47" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D47" t="s">
         <v>37</v>
@@ -2510,10 +2507,10 @@
     </row>
     <row r="48" spans="1:7" ht="116" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C48" t="s">
         <v>21</v>
@@ -2530,10 +2527,10 @@
     </row>
     <row r="49" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C49" t="s">
         <v>21</v>
@@ -2544,10 +2541,10 @@
     </row>
     <row r="50" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B50" s="3" t="s">
         <v>200</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>201</v>
       </c>
       <c r="C50" t="s">
         <v>21</v>
@@ -2564,10 +2561,10 @@
     </row>
     <row r="51" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C51" t="s">
         <v>21</v>
@@ -2587,10 +2584,10 @@
     </row>
     <row r="52" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A52" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C52" t="s">
         <v>21</v>
@@ -2610,10 +2607,10 @@
     </row>
     <row r="53" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A53" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C53" t="s">
         <v>21</v>
@@ -2633,10 +2630,10 @@
     </row>
     <row r="54" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A54" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C54" t="s">
         <v>21</v>
@@ -2656,10 +2653,10 @@
     </row>
     <row r="55" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C55" t="s">
         <v>21</v>
@@ -2679,10 +2676,10 @@
     </row>
     <row r="56" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A56" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C56" t="s">
         <v>21</v>
@@ -2702,10 +2699,10 @@
     </row>
     <row r="57" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C57" t="s">
         <v>21</v>
@@ -2725,10 +2722,10 @@
     </row>
     <row r="58" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C58" t="s">
         <v>21</v>
@@ -2748,10 +2745,10 @@
     </row>
     <row r="59" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C59" t="s">
         <v>21</v>
@@ -2774,7 +2771,7 @@
         <v>31</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C60" t="s">
         <v>21</v>
@@ -2797,7 +2794,7 @@
         <v>110</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C61" t="s">
         <v>21</v>
@@ -2820,7 +2817,7 @@
         <v>116</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C62" t="s">
         <v>21</v>
@@ -2843,7 +2840,7 @@
         <v>112</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C63" t="s">
         <v>21</v>
@@ -2866,7 +2863,7 @@
         <v>117</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C64" t="s">
         <v>21</v>
@@ -2889,7 +2886,7 @@
         <v>121</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C65" t="s">
         <v>21</v>
@@ -2906,7 +2903,7 @@
         <v>125</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C66" t="s">
         <v>21</v>
@@ -2923,7 +2920,7 @@
         <v>126</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C67" t="s">
         <v>21</v>
@@ -2937,10 +2934,10 @@
     </row>
     <row r="68" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B68" s="3" t="s">
         <v>241</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>242</v>
       </c>
       <c r="C68" t="s">
         <v>21</v>
@@ -2963,13 +2960,13 @@
         <v>170</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C69" t="s">
         <v>21</v>
       </c>
       <c r="D69" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E69" t="s">
         <v>172</v>
@@ -3222,27 +3219,27 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="49" spans="2:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="50" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="51" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B51" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="52" spans="2:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B52" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -3264,6 +3261,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="985d26ac-cf7b-4687-94e0-26b141782da7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100527ED9A1E2F34D48AA5925CCBA0CEC41" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="73c2da0cd5c8d9fd369ff3018c825410">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4" xmlns:ns3="985d26ac-cf7b-4687-94e0-26b141782da7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b3600b0f37fd05e6cabe55b41d10e7dc" ns2:_="" ns3:_="">
     <xsd:import namespace="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4"/>
@@ -3458,17 +3466,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="985d26ac-cf7b-4687-94e0-26b141782da7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12DB76A7-ED98-4EE3-9432-17F601352CF4}">
   <ds:schemaRefs>
@@ -3478,6 +3475,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E61FE636-68A4-4725-8134-F4B9672BB2E7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="985d26ac-cf7b-4687-94e0-26b141782da7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9675DCA-D684-4E4E-B61D-0AB2D6821582}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3494,21 +3508,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E61FE636-68A4-4725-8134-F4B9672BB2E7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="985d26ac-cf7b-4687-94e0-26b141782da7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Updated and added mappings and code
</commit_message>
<xml_diff>
--- a/Map/USDM2FHIR.xlsx
+++ b/Map/USDM2FHIR.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\USDM_db\Map\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDE9255-A218-4184-A17D-0B729E65BE66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864766BC-2522-404A-85B4-A39425393F66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-11700" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{97BCDFE6-590C-45E1-8F75-1AA7EE2945FF}"/>
+    <workbookView xWindow="-4545" yWindow="-16080" windowWidth="26250" windowHeight="14925" xr2:uid="{97BCDFE6-590C-45E1-8F75-1AA7EE2945FF}"/>
   </bookViews>
   <sheets>
     <sheet name="USDM2FHIR map" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="335">
   <si>
     <t>Item</t>
   </si>
@@ -217,12 +217,6 @@
     <t>study.versions.studyDesigns.objectives[level.code="C163559"].{id: "Exploratory"}</t>
   </si>
   <si>
-    <t>Endpoints</t>
-  </si>
-  <si>
-    <t>objective.outcomeMeasure.name</t>
-  </si>
-  <si>
     <t>objective;outcomeMeasure</t>
   </si>
   <si>
@@ -247,9 +241,6 @@
     <t>USDM path instructions:</t>
   </si>
   <si>
-    <t>The path must incldue the full USDM json path starting at the study level.</t>
-  </si>
-  <si>
     <t>The results must include an id value and a corresponding result value. The id value can be used to group information from different mappings between entries. Mapping at the end should be like: {id: ….}</t>
   </si>
   <si>
@@ -274,9 +265,6 @@
     <t>study.versions.studyDesigns.objectives@$ob.$ob.endpoints.{$ob.id: text}</t>
   </si>
   <si>
-    <t>phase</t>
-  </si>
-  <si>
     <t>Include id for groupings of nested information at the highhest level. E.g. the id for objectives should be used in the objectives/endpoints combinations.</t>
   </si>
   <si>
@@ -295,9 +283,6 @@
     <t>Study Identifier Organization</t>
   </si>
   <si>
-    <t>study.versions.studyIdentifiers[$substring(text,0,3)="NCT"].{id: "https://clinicaltrials.gov"}</t>
-  </si>
-  <si>
     <t>NCT identifier system</t>
   </si>
   <si>
@@ -328,48 +313,9 @@
     <t>site country</t>
   </si>
   <si>
-    <t>study.versions.studyDesigns.population[includesHealthySubjects=false].{id: "Does not include healthy volunteers"}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.population[includesHealthySubjects=false].{id: "does-not-include-healthy-volunteers"}</t>
-  </si>
-  <si>
-    <t>no healthy subjects code</t>
-  </si>
-  <si>
-    <t>no healthy subjects decode</t>
-  </si>
-  <si>
-    <t>healthy subjects code</t>
-  </si>
-  <si>
-    <t>healthy subjects decode</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.population[includesHealthySubjects=true].{id: "includes-healthy-volunteers"}</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.population[includesHealthySubjects=true].{id: "Includes healthy volunteers"}</t>
-  </si>
-  <si>
-    <t>classifier.coding.code</t>
-  </si>
-  <si>
-    <t>classifier.coding.display</t>
-  </si>
-  <si>
-    <t>(no) healthy subjects codeSystem</t>
-  </si>
-  <si>
-    <t>study.versions.studyDesigns.population.{id: "https://fevir.net/resources/CodeSystem/419455"}</t>
-  </si>
-  <si>
     <t>purposeType</t>
   </si>
   <si>
-    <t>classifier.coding.system</t>
-  </si>
-  <si>
     <t>classifier.text</t>
   </si>
   <si>
@@ -535,9 +481,6 @@
     <t>Extenstion url's:</t>
   </si>
   <si>
-    <t>USDM Extensions need a url to indicate the extended class or attribute. If the url name changes, this needs to be changed in the JSONata mappings as well. The following url's are used in the mappings:</t>
-  </si>
-  <si>
     <t>The class in USDM in which the information is stored</t>
   </si>
   <si>
@@ -566,9 +509,6 @@
   </si>
   <si>
     <t>The FHIR resource that the item maps to. Initially either StudyDefinition for the general study design information or Group for the expected response information.</t>
-  </si>
-  <si>
-    <t>The FHIR json level used to index multiple results within 1 mapping to allow for subgrouping.</t>
   </si>
   <si>
     <t>If an aliasCode datatype is available in USDM then adding the correct FHIR coding as an aliascode at the source is more efficient and clear in lineage than including it in the mapping. See for example StudyPhase mapping which assumes the storage of the corresponding FHIR code in USDM. For the Biomedical concepts the corresponding LOINC code must be included in USDM as an alias.</t>
@@ -628,13 +568,6 @@
   $sv.studyDesigns.eligibilityCriteria@$ex.(
   $respIds := $sv.extensionAttributes.extensionAttributes.valueExtensionClass[url="https://cdisc.org/usdm/extension-ExpResponse/class_ExpectedResponse" and extensionAttributes[valueId=$ex.id]].id;
   {$ex.id: ($respIds) ? "Group"}))</t>
-  </si>
-  <si>
-    <t>study.versions@$sv.(
-  $sv.studyDesigns.eligibilityCriteria@$ex.(
-  $respIds := $sv.extensionAttributes.extensionAttributes.valueExtensionClass[url="https://cdisc.org/usdm/extension-ExpResponse/class_ExpectedResponse" and extensionAttributes[valueId=$ex.id]].id;
-  $nodeIds := $sv.extensionAttributes.extensionAttributes.valueExtensionClass[url="https://cdisc.org/usdm/extension-ExpResponseNode/class1" and extensionAttributes.extensionAttributes[valueId in $respIds]].id;
-  {$ex.id: $nodeIds ? $nodeIds : $respIds}))</t>
   </si>
   <si>
     <t>study.versions@$sv.(
@@ -754,9 +687,6 @@
   </si>
   <si>
     <t>expected response description</t>
-  </si>
-  <si>
-    <t>Tooling limits</t>
   </si>
   <si>
     <t>The tool is a MVP. Therefore it does not cover all potential complexities and the output should be carefully validated before use.</t>
@@ -965,12 +895,6 @@
 {id: {"code": code, "display": decode, "system": codeSystem}}</t>
   </si>
   <si>
-    <t>study.versions.studyDesigns.intentTypes.(
-    $FCod := function($c){$replace($lowercase($c), " ", "-")};
-    $titleCase := function($s) {$join($split($lowercase($s), " ")@$w.($uppercase($substring($w, 0, 1)) &amp; $substring($w, 1))," ")};
-{id: {"code": $FCod(decode), "display": $titleCase(decode), "system": "http://terminology.hl7.org/CodeSystem/research-study-prim-purp-type"}})</t>
-  </si>
-  <si>
     <t>purposeType.coding</t>
   </si>
   <si>
@@ -992,9 +916,6 @@
     <t>label.type.coding</t>
   </si>
   <si>
-    <t>study.versions.studyDesigns.indications.{id: {"code": codes.code, "display": codes.decode, "system": codes.codeSystem, "version": codes.codeSystemVersion}}</t>
-  </si>
-  <si>
     <t>condition.coding</t>
   </si>
   <si>
@@ -1027,9 +948,6 @@
     <t>label.language</t>
   </si>
   <si>
-    <t>purpose _ intent</t>
-  </si>
-  <si>
     <t>study.versions.studyDesigns.objectives@$ob.$ob.endpoints.(
     $firstWord := function($s) {$split($s, " ")[0]};
     $titleCase := function($s) {$join($split($lowercase($s), " ")@$w.($uppercase($substring($w, 0, 1)) &amp; $substring($w, 1))," ")};
@@ -1082,13 +1000,300 @@
     <t>startDate, endDate</t>
   </si>
   <si>
-    <t>{"eligibility-criteria": {"reference": "eligibility-criteria", "type":"Group"}}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">study.versions.organizations.managedSites.{id: {"reference": id, "type":"Location"}} </t>
-  </si>
-  <si>
     <t>(study.versions)@$sv.$sv.studyIdentifiers@$id.$id{id: $sv.organizations[id=$id.scopeId].label}</t>
+  </si>
+  <si>
+    <t>USDM Extensions need a url to indicate the extended class or attribute. Note that these url's are still draft and need to be changed upon finalization. If the url name changes, this needs to be changed in the JSONata mappings as well. The following url's are used in the mappings:</t>
+  </si>
+  <si>
+    <t>Code system references</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FHIR uses standard system uri references which are noted in https://terminology.hl7.org/en/external_code_systems.html  </t>
+  </si>
+  <si>
+    <t>These references are recommended to be used directly when creating USDM in case a related codesystem is referenced.</t>
+  </si>
+  <si>
+    <t>For example in an alias code, study indication or extension reference</t>
+  </si>
+  <si>
+    <t>"C16576" in study.versions.studyDesigns.population.plannedSex.code ? {"f01": {"coding": {
+        "code": "includes-females",
+        "display": "Includes female subjects",
+        "system": "https://fevir.net/resources/CodeSystem/419455"
+      }}} : " "</t>
+  </si>
+  <si>
+    <t>"C20197" in study.versions.studyDesigns.population.plannedSex.code ? {"m01": {"coding": {
+        "code": "includes-males",
+        "display": "Includes male subjects",
+        "system": "https://fevir.net/resources/CodeSystem/419455"
+      }}} : " "</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.population[includesHealthySubjects=false].{id: {"coding": {
+        "code": "does-not-include-healthy-volunteers",
+        "display": "Does not include healthy volunteers",
+        "system": "https://fevir.net/resources/CodeSystem/419455"
+      }}}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.population[includesHealthySubjects=true].{id: {"coding": {
+        "code": "includes-healthy-volunteers",
+        "display": "Includes healthy volunteers",
+        "system": "https://fevir.net/resources/CodeSystem/419455"
+      }}}</t>
+  </si>
+  <si>
+    <t>PlannedSex</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.population.plannedAge[minValue.value&lt;18 and minValue.unit.standardCode.code="C29848"].{id: {"coding": {
+        "code": "includes-ages-0-17",
+        "display": "Includes ages 0-17 years",
+        "system": "https://fevir.net/resources/CodeSystem/419455"
+      }}}</t>
+  </si>
+  <si>
+    <t>Includes females code (cohort definitions not included)</t>
+  </si>
+  <si>
+    <t>Includes males code (cohort definitions not included)</t>
+  </si>
+  <si>
+    <t>no healthy subjects code (cohort definitions not included)</t>
+  </si>
+  <si>
+    <t>healthy subjects code (cohort definitions not included)</t>
+  </si>
+  <si>
+    <t>age category 0-17 (Only based on population and year unit)</t>
+  </si>
+  <si>
+    <t>age category 18-64 (Only based on population and year unit)</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.population.plannedAge[(minValue.value&lt;65 and minValue.unit.standardCode.code="C29848") and (maxValue.value&gt;17 and maxValue.unit.standardCode.code="C29848") ].{id&amp;"b": {"coding": {
+        "code": "includes-ages-18-64",
+        "display": "Includes ages 18-64 years",
+        "system": "https://fevir.net/resources/CodeSystem/419455"
+      }}}</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.population.plannedAge[(maxValue.value&gt;64 and maxValue.unit.standardCode.code="C29848")].{id&amp;"c": {"coding": {
+        "code": "includes-ages-65-and-older",
+        "display": "Includes ages 65 and older",
+        "system": "https://fevir.net/resources/CodeSystem/419455"
+      }}}</t>
+  </si>
+  <si>
+    <t>age category 65 and older (Only based on population and year unit)</t>
+  </si>
+  <si>
+    <t>FHIR classifiers are mapped as indicated in https://fevir.net/resources/CodeSystem/419455</t>
+  </si>
+  <si>
+    <t>FHIR Classifiers</t>
+  </si>
+  <si>
+    <t>The path must include the full USDM json path starting at the study level.</t>
+  </si>
+  <si>
+    <t>Run statement for the tooling: python CreateFhir.py --map Map/USDM2FHIR.csv --usdm Input/NCT01750580_limited_tagged_resp.json --output Output/MyNewFile.json</t>
+  </si>
+  <si>
+    <t>Tool limits</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.indications.{id: {"code": codes.code, "display": codes.decode, "system": codes.codeSystem}}</t>
+  </si>
+  <si>
+    <t>study.versions.studyIdentifiers[$substring(text,0,3)="NCT"].{id: "http://terminology.hl7.org/NamingSystem/ClinicalTrials-Gov"}</t>
+  </si>
+  <si>
+    <t>Study Identifier FHIR type</t>
+  </si>
+  <si>
+    <t>study.versions.studyIdentifiers.{id: "study identifier"}</t>
+  </si>
+  <si>
+    <t>identifier.codeableConcept.text</t>
+  </si>
+  <si>
+    <t>The FHIR json level used to index multiple results within 1 mapping to allow for subgrouping. Leave empty in case the result in FHIR should not be stored as an array on any level!!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">study.versions.organizations.managedSites.{id: {"reference": "#" &amp; id, "type":"Location"}} </t>
+  </si>
+  <si>
+    <t>{"eligibility-criteria": {"reference": "#eligibility-criteria", "type":"Group"}}</t>
+  </si>
+  <si>
+    <t>study.versions@$sv.(
+  $sv.studyDesigns.eligibilityCriteria@$ex.(
+  $respIds := $sv.extensionAttributes.extensionAttributes.valueExtensionClass[url="https://cdisc.org/usdm/extension-ExpResponse/class_ExpectedResponse" and extensionAttributes[valueId=$ex.id]].("#"&amp; id);
+  $nodeIds := $sv.extensionAttributes.extensionAttributes.valueExtensionClass[url="https://cdisc.org/usdm/extension-ExpResponseNode/class1" and extensionAttributes.extensionAttributes["#" &amp; valueId in $respIds]].("#" &amp; id);
+  {$ex.id: $nodeIds ? $nodeIds : $respIds}))</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.intentTypes.(
+    $Recode := function($c){$c="C49656" ? "treatment" : $c="C49657" ? "prevention" : $c="C49653" ? "diagnostic" : $c="C71485" ? "screening" :
+        $c="C71486" ? "supportive-care" : $c="C15245" ? "health-services-research" : $c="C15714" ? "basic-science" : $c="C139174" ? "device-feasibility"};
+    $RecodeDisplay := function($c){$c="C49656" ? "Treatment Study" : $c="C49657" ? "Prevention Study" : $c="C49653" ? "Diagnostic Study" : $c="C71485" ? "Screening Study" :
+        $c="C71486" ? "Supportive Care Study" : $c="C15245" ? "Health Services Research" : $c="C15714" ? "Basic Science" : $c="C139174" ? "Device Feasibility Study"};
+{id: {"code": $Recode(code), "display": $RecodeDisplay(code), "system": "http://terminology.hl7.org/CodeSystem/research-study-purpose-type"}})</t>
+  </si>
+  <si>
+    <t>purpose Intent</t>
+  </si>
+  <si>
+    <t>purpose SubType</t>
+  </si>
+  <si>
+    <t>InterventionalStudyDesign</t>
+  </si>
+  <si>
+    <t>intentTypes</t>
+  </si>
+  <si>
+    <t>subTypes</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.subTypes.(
+    $Recode := function($c){$c="C49667" ? "safety" : $c="C49666" ? "efficacy" : $c="C49663" ? "pharmacokinetic" : 
+                            $c="C49662" ? "pharmacodynamic" : $c="C49665" ? "bioequivalence" : $c="C127803" ? "dose-response" : 
+                            $c="C129001" ? "pharmacogenetic" : $c="C49661" ? "pharmacogenomic" : $c="C215653" ? "incidence" : 
+                            $c="C215675" ? "prevalence"};
+    $RecodeDisplay := function($c){$c="C49667" ? "Safety Study" : $c="C49666" ? "Efficacy Study" : $c="C49663" ? "Pharmacokinetic Study" : 
+                            $c="C49662" ? "Pharmacodynamic Study" : $c="C49665" ? "Bioequivalence Study" : $c="C127803" ? "Dose-Response Study" : 
+                            $c="C129001" ? "Pharmacogenetic Study" : $c="C49661" ? "Pharmacogenomic Study": $c="C215653" ? "Incidence Study" : 
+                            $c="C215675" ? "Prevalence Study"}
+{id: $Recode(code) ? {"code": $Recode(code), "display": $RecodeDisplay(code), "system": "http://terminology.hl7.org/CodeSystem/research-study-purpose-type"}
+ : {"text": decode}})</t>
+  </si>
+  <si>
+    <t>objective.outcomeMeasure.endpoint.display</t>
+  </si>
+  <si>
+    <t>Evidence variable id</t>
+  </si>
+  <si>
+    <t>EvidenceVariable</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives@$ob.$ob.endpoints.(
+    $bcId := extensionAttributes[url="https://cdisc.org/usdm/extension-ExpResponse-1/attribute-relatedAssessment"].valueId;
+    {$bcId: $bcId })</t>
+  </si>
+  <si>
+    <t>Evidence variable name</t>
+  </si>
+  <si>
+    <t>study.versions@$sv.$sv.studyDesigns.objectives@$ob.$ob.endpoints.(
+    $bcId := extensionAttributes[url="https://cdisc.org/usdm/extension-ExpResponse-1/attribute-relatedAssessment"].valueId;
+    {$bcId: $sv.biomedicalConcepts[id=$bcId].name })</t>
+  </si>
+  <si>
+    <t>Evidence variable title</t>
+  </si>
+  <si>
+    <t>study.versions@$sv.$sv.studyDesigns.objectives@$ob.$ob.endpoints.(
+    $bcId := extensionAttributes[url="https://cdisc.org/usdm/extension-ExpResponse-1/attribute-relatedAssessment"].valueId;
+    {$bcId: $sv.biomedicalConcepts[id=$bcId].label })</t>
+  </si>
+  <si>
+    <t>study.versions@$sv.$sv.studyDesigns.objectives@$ob.$ob.endpoints.(
+    $bcId := extensionAttributes[url="https://cdisc.org/usdm/extension-ExpResponse-1/attribute-relatedAssessment"].valueId;
+    {$bcId: $sv.biomedicalConcepts[id=$bcId].description })</t>
+  </si>
+  <si>
+    <t>Evidence variable description</t>
+  </si>
+  <si>
+    <t>study.versions@$sv.$sv.studyDesigns.objectives@$ob.$ob.endpoints.(
+    $bcId := extensionAttributes[url="https://cdisc.org/usdm/extension-ExpResponse-1/attribute-relatedAssessment"].valueId;
+    {$bcId: {"code" : "measurement", "display": "Measurement", "system": "http://hl7.org/fhir/evidence-variable-classifier-example"} })</t>
+  </si>
+  <si>
+    <t>Evidence classifier (note that questionnaires should get another code / not taken care of yet)</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.objectives@$ob.$ob.endpoints.(
+    $bcId := extensionAttributes[url="https://cdisc.org/usdm/extension-ExpResponse-1/attribute-relatedAssessment"].valueId;
+    {$ob.id: $bcId ? {"reference": "#" &amp; extensionAttributes[url="https://cdisc.org/usdm/extension-ExpResponse-1/attribute-relatedAssessment"].valueId, "type": "EvidenceVariable" }})</t>
+  </si>
+  <si>
+    <t>Outcome measurement display</t>
+  </si>
+  <si>
+    <t>Outcome measurement reference or display</t>
+  </si>
+  <si>
+    <t>objective.outcomeMeasure.endpoint</t>
+  </si>
+  <si>
+    <t>Eligibility criteria code</t>
+  </si>
+  <si>
+    <t>characteristic.code.text</t>
+  </si>
+  <si>
+    <t>EligibilityCriterionItem</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.eligibilityCriteria.{id: label}</t>
+  </si>
+  <si>
+    <t>Arm name</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.arms.label</t>
+  </si>
+  <si>
+    <t>comparisonGroup</t>
+  </si>
+  <si>
+    <t>comparisonGroup.name</t>
+  </si>
+  <si>
+    <t>StudyArm</t>
+  </si>
+  <si>
+    <t>Arm description</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.arms.description</t>
+  </si>
+  <si>
+    <t>comparisonGroup.description</t>
+  </si>
+  <si>
+    <t>Cohort name</t>
+  </si>
+  <si>
+    <t>Cohort description</t>
+  </si>
+  <si>
+    <t>Cohort planned number</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.population.cohorts.label</t>
+  </si>
+  <si>
+    <t>studyCohort</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.population.cohorts.description</t>
+  </si>
+  <si>
+    <t>study.versions.studyDesigns.population.cohorts.plannedEnrollmentNumber.value</t>
+  </si>
+  <si>
+    <t>comparisonGroup.targetNumber</t>
+  </si>
+  <si>
+    <t>plannedEnrollmentNumber</t>
   </si>
 </sst>
 </file>
@@ -1154,7 +1359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1174,6 +1379,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1508,7 +1714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81DD2990-A668-4ED7-89E0-40F5440ED267}">
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.1796875" style="3" customWidth="1"/>
@@ -1525,7 +1731,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>20</v>
@@ -1537,10 +1743,10 @@
         <v>42</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
@@ -1551,7 +1757,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -1560,7 +1766,7 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="G2" t="s">
         <v>9</v>
@@ -1571,33 +1777,33 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>255</v>
+        <v>282</v>
       </c>
       <c r="C3" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D3" t="s">
-        <v>256</v>
+        <v>232</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
       </c>
       <c r="F3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="G3" t="s">
-        <v>132</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>244</v>
+        <v>222</v>
       </c>
       <c r="C4" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -1606,1388 +1812,1715 @@
         <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="G4" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>83</v>
+        <v>284</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C5" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>286</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>133</v>
-      </c>
-      <c r="G5" t="s">
-        <v>135</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>84</v>
+        <v>256</v>
       </c>
       <c r="C6" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D6" t="s">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
         <v>10</v>
       </c>
+      <c r="F6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G6" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>243</v>
+        <v>80</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>242</v>
+        <v>283</v>
       </c>
       <c r="C7" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D7" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
       </c>
+      <c r="F7" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
+        <v>221</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>220</v>
       </c>
       <c r="C8" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D8" t="s">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="E8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" t="s">
-        <v>136</v>
-      </c>
-      <c r="G8" t="s">
-        <v>134</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D9" t="s">
-        <v>81</v>
+        <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
       <c r="F9" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="G9" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>253</v>
+        <v>76</v>
+      </c>
+      <c r="B10" t="s">
+        <v>75</v>
       </c>
       <c r="C10" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D10" t="s">
-        <v>254</v>
-      </c>
-      <c r="E10" t="s">
-        <v>9</v>
+        <v>77</v>
       </c>
       <c r="F10" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="G10" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>257</v>
+        <v>229</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>258</v>
+        <v>230</v>
       </c>
       <c r="C11" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D11" t="s">
-        <v>8</v>
+        <v>231</v>
       </c>
       <c r="E11" t="s">
         <v>9</v>
       </c>
       <c r="F11" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="G11" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>260</v>
+        <v>233</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>261</v>
+        <v>234</v>
       </c>
       <c r="C12" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D12" t="s">
-        <v>254</v>
+        <v>8</v>
       </c>
       <c r="E12" t="s">
         <v>9</v>
       </c>
       <c r="F12" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="G12" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>262</v>
+        <v>236</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>263</v>
+        <v>237</v>
       </c>
       <c r="C13" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D13" t="s">
-        <v>264</v>
+        <v>231</v>
       </c>
       <c r="E13" t="s">
         <v>9</v>
       </c>
       <c r="F13" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="G13" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>16</v>
+        <v>238</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>15</v>
+        <v>239</v>
       </c>
       <c r="C14" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D14" t="s">
-        <v>109</v>
+        <v>240</v>
       </c>
       <c r="E14" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="F14" t="s">
-        <v>141</v>
+        <v>118</v>
       </c>
       <c r="G14" t="s">
-        <v>138</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D15" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="E15" t="s">
         <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="G15" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="C16" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D16" t="s">
-        <v>39</v>
+        <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="G16" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>43</v>
+        <v>268</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>51</v>
+        <v>262</v>
       </c>
       <c r="C17" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D17" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="E17" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="F17" t="s">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="G17" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>43</v>
+        <v>269</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>52</v>
+        <v>263</v>
       </c>
       <c r="C18" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D18" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E18" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="F18" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="G18" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>44</v>
+        <v>270</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>53</v>
+        <v>264</v>
       </c>
       <c r="C19" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D19" t="s">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="E19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+      <c r="F19" t="s">
+        <v>129</v>
+      </c>
+      <c r="G19" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
-        <v>48</v>
+        <v>271</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>54</v>
+        <v>265</v>
       </c>
       <c r="C20" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D20" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="E20" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="F20" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="G20" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>48</v>
+        <v>272</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>55</v>
+        <v>267</v>
       </c>
       <c r="C21" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D21" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E21" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="F21" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="G21" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>49</v>
+        <v>273</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>56</v>
+        <v>274</v>
       </c>
       <c r="C22" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D22" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="E22" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="F22" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="G22" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
-        <v>49</v>
+        <v>276</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>57</v>
+        <v>275</v>
       </c>
       <c r="C23" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D23" t="s">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="E23" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="F23" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="G23" t="s">
-        <v>140</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="C24" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D24" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="E24" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F24" t="s">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="G24" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
-        <v>250</v>
+        <v>43</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>266</v>
+        <v>51</v>
       </c>
       <c r="C25" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D25" t="s">
-        <v>251</v>
+        <v>45</v>
       </c>
       <c r="E25" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F25" t="s">
-        <v>142</v>
+        <v>121</v>
       </c>
       <c r="G25" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="58" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>265</v>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="3" t="s">
+        <v>43</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>248</v>
+        <v>52</v>
       </c>
       <c r="C26" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D26" t="s">
-        <v>249</v>
+        <v>46</v>
       </c>
       <c r="E26" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+      <c r="F26" t="s">
+        <v>121</v>
+      </c>
+      <c r="G26" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>246</v>
+        <v>44</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>247</v>
+        <v>53</v>
       </c>
       <c r="C27" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D27" t="s">
-        <v>245</v>
+        <v>47</v>
       </c>
       <c r="E27" t="s">
-        <v>77</v>
-      </c>
-      <c r="F27" t="s">
-        <v>143</v>
-      </c>
-      <c r="G27" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="3" t="s">
-        <v>267</v>
+        <v>48</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>276</v>
+        <v>54</v>
       </c>
       <c r="C28" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D28" t="s">
-        <v>268</v>
+        <v>45</v>
       </c>
       <c r="E28" t="s">
-        <v>269</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+      <c r="F28" t="s">
+        <v>121</v>
+      </c>
+      <c r="G28" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
-        <v>272</v>
+        <v>48</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>277</v>
+        <v>55</v>
       </c>
       <c r="C29" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D29" t="s">
-        <v>273</v>
+        <v>46</v>
       </c>
       <c r="E29" t="s">
-        <v>269</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="G29" s="7" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>40</v>
+      </c>
+      <c r="F29" t="s">
+        <v>121</v>
+      </c>
+      <c r="G29" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="3" t="s">
-        <v>275</v>
+        <v>49</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>278</v>
+        <v>56</v>
       </c>
       <c r="C30" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D30" t="s">
-        <v>279</v>
+        <v>45</v>
       </c>
       <c r="E30" t="s">
-        <v>269</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>280</v>
+        <v>40</v>
+      </c>
+      <c r="F30" t="s">
+        <v>121</v>
+      </c>
+      <c r="G30" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="3" t="s">
-        <v>232</v>
+        <v>49</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>282</v>
+        <v>57</v>
       </c>
       <c r="C31" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D31" t="s">
+        <v>46</v>
+      </c>
+      <c r="E31" t="s">
+        <v>40</v>
+      </c>
+      <c r="F31" t="s">
+        <v>121</v>
+      </c>
+      <c r="G31" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="58" x14ac:dyDescent="0.35">
+      <c r="A32" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="C32" t="s">
+        <v>161</v>
+      </c>
+      <c r="D32" t="s">
+        <v>313</v>
+      </c>
+      <c r="E32" t="s">
+        <v>58</v>
+      </c>
+      <c r="F32" t="s">
+        <v>124</v>
+      </c>
+      <c r="G32" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A33" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" t="s">
+        <v>161</v>
+      </c>
+      <c r="D33" t="s">
+        <v>298</v>
+      </c>
+      <c r="E33" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C34" t="s">
+        <v>161</v>
+      </c>
+      <c r="D34" t="s">
+        <v>228</v>
+      </c>
+      <c r="E34" t="s">
+        <v>58</v>
+      </c>
+      <c r="F34" t="s">
+        <v>124</v>
+      </c>
+      <c r="G34" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>292</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="C35" t="s">
+        <v>161</v>
+      </c>
+      <c r="D35" t="s">
+        <v>226</v>
+      </c>
+      <c r="E35" t="s">
         <v>90</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F35" t="s">
+        <v>294</v>
+      </c>
+      <c r="G35" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+      <c r="A36" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="C36" t="s">
+        <v>161</v>
+      </c>
+      <c r="D36" t="s">
+        <v>226</v>
+      </c>
+      <c r="E36" t="s">
         <v>90</v>
       </c>
-      <c r="F31" t="s">
-        <v>145</v>
-      </c>
-      <c r="G31" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>231</v>
-      </c>
-      <c r="C32" t="s">
-        <v>234</v>
-      </c>
-      <c r="D32" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C33" t="s">
-        <v>234</v>
-      </c>
-      <c r="D33" t="s">
-        <v>235</v>
-      </c>
-      <c r="F33" t="s">
-        <v>145</v>
-      </c>
-      <c r="G33" t="s">
+      <c r="F36" t="s">
+        <v>294</v>
+      </c>
+      <c r="G36" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A37" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C37" t="s">
+        <v>161</v>
+      </c>
+      <c r="D37" t="s">
+        <v>223</v>
+      </c>
+      <c r="F37" t="s">
+        <v>125</v>
+      </c>
+      <c r="G37" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A38" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="C38" t="s">
+        <v>161</v>
+      </c>
+      <c r="D38" t="s">
+        <v>243</v>
+      </c>
+      <c r="E38" t="s">
+        <v>244</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A39" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="C39" t="s">
+        <v>161</v>
+      </c>
+      <c r="D39" t="s">
+        <v>248</v>
+      </c>
+      <c r="E39" t="s">
+        <v>244</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A40" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="C40" t="s">
+        <v>161</v>
+      </c>
+      <c r="D40" t="s">
+        <v>254</v>
+      </c>
+      <c r="E40" t="s">
+        <v>244</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C41" t="s">
+        <v>161</v>
+      </c>
+      <c r="D41" t="s">
+        <v>321</v>
+      </c>
+      <c r="E41" t="s">
+        <v>320</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="G41" s="9" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C34" t="s">
-        <v>234</v>
-      </c>
-      <c r="D34" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C35" t="s">
-        <v>234</v>
-      </c>
-      <c r="D35" t="s">
-        <v>236</v>
-      </c>
-      <c r="F35" t="s">
-        <v>145</v>
-      </c>
-      <c r="G35" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A36" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C36" t="s">
-        <v>181</v>
-      </c>
-      <c r="D36" t="s">
-        <v>103</v>
-      </c>
-      <c r="E36" t="s">
-        <v>19</v>
-      </c>
-      <c r="F36" t="s">
-        <v>147</v>
-      </c>
-      <c r="G36" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A37" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="C37" t="s">
-        <v>181</v>
-      </c>
-      <c r="D37" t="s">
-        <v>104</v>
-      </c>
-      <c r="E37" t="s">
-        <v>19</v>
-      </c>
-      <c r="F37" t="s">
-        <v>147</v>
-      </c>
-      <c r="G37" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A38" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C38" t="s">
-        <v>181</v>
-      </c>
-      <c r="D38" t="s">
-        <v>103</v>
-      </c>
-      <c r="E38" t="s">
-        <v>19</v>
-      </c>
-      <c r="F38" t="s">
-        <v>147</v>
-      </c>
-      <c r="G38" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A39" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="C39" t="s">
-        <v>181</v>
-      </c>
-      <c r="D39" t="s">
-        <v>104</v>
-      </c>
-      <c r="E39" t="s">
-        <v>19</v>
-      </c>
-      <c r="F39" t="s">
-        <v>147</v>
-      </c>
-      <c r="G39" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A40" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C40" t="s">
-        <v>181</v>
-      </c>
-      <c r="D40" t="s">
-        <v>108</v>
-      </c>
-      <c r="E40" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A41" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="C41" t="s">
-        <v>181</v>
-      </c>
-      <c r="D41" t="s">
-        <v>228</v>
-      </c>
-      <c r="E41" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="3" t="s">
-        <v>182</v>
+        <v>323</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>183</v>
+        <v>324</v>
       </c>
       <c r="C42" t="s">
-        <v>186</v>
+        <v>161</v>
       </c>
       <c r="D42" t="s">
-        <v>38</v>
+        <v>325</v>
+      </c>
+      <c r="E42" t="s">
+        <v>320</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A43" s="3" t="s">
-        <v>189</v>
+        <v>326</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>188</v>
+        <v>329</v>
       </c>
       <c r="C43" t="s">
-        <v>186</v>
+        <v>161</v>
       </c>
       <c r="D43" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+        <v>321</v>
+      </c>
+      <c r="E43" t="s">
+        <v>320</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A44" s="3" t="s">
-        <v>184</v>
+        <v>327</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>185</v>
+        <v>331</v>
       </c>
       <c r="C44" t="s">
-        <v>186</v>
+        <v>161</v>
       </c>
       <c r="D44" t="s">
-        <v>27</v>
+        <v>325</v>
       </c>
       <c r="E44" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+        <v>320</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="3" t="s">
-        <v>169</v>
+        <v>328</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>187</v>
+        <v>332</v>
       </c>
       <c r="C45" t="s">
-        <v>186</v>
+        <v>161</v>
       </c>
       <c r="D45" t="s">
-        <v>152</v>
+        <v>333</v>
       </c>
       <c r="E45" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
+        <v>320</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="3" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>194</v>
+        <v>288</v>
       </c>
       <c r="C46" t="s">
-        <v>186</v>
+        <v>161</v>
       </c>
       <c r="D46" t="s">
-        <v>35</v>
+        <v>85</v>
       </c>
       <c r="E46" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+        <v>85</v>
+      </c>
+      <c r="F46" t="s">
+        <v>127</v>
+      </c>
+      <c r="G46" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" s="3" t="s">
-        <v>36</v>
+        <v>211</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
       <c r="C47" t="s">
-        <v>186</v>
+        <v>212</v>
       </c>
       <c r="D47" t="s">
-        <v>37</v>
-      </c>
-      <c r="E47" t="s">
-        <v>172</v>
-      </c>
-      <c r="F47" t="s">
-        <v>149</v>
-      </c>
-      <c r="G47" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" ht="116" x14ac:dyDescent="0.35">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="3" t="s">
-        <v>196</v>
+        <v>84</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>195</v>
+        <v>83</v>
       </c>
       <c r="C48" t="s">
-        <v>21</v>
+        <v>212</v>
       </c>
       <c r="D48" t="s">
-        <v>38</v>
+        <v>213</v>
       </c>
       <c r="F48" t="s">
-        <v>149</v>
+        <v>127</v>
       </c>
       <c r="G48" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A49" s="3" t="s">
-        <v>198</v>
+        <v>86</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>197</v>
+        <v>87</v>
       </c>
       <c r="C49" t="s">
-        <v>21</v>
+        <v>212</v>
       </c>
       <c r="D49" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A50" s="3" t="s">
-        <v>199</v>
+        <v>89</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>200</v>
+        <v>88</v>
       </c>
       <c r="C50" t="s">
-        <v>21</v>
+        <v>212</v>
       </c>
       <c r="D50" t="s">
-        <v>22</v>
+        <v>214</v>
       </c>
       <c r="F50" t="s">
-        <v>149</v>
+        <v>127</v>
       </c>
       <c r="G50" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>207</v>
       </c>
       <c r="B51" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C51" t="s">
+        <v>161</v>
+      </c>
+      <c r="D51" t="s">
         <v>206</v>
       </c>
-      <c r="C51" t="s">
-        <v>21</v>
-      </c>
-      <c r="D51" t="s">
-        <v>23</v>
-      </c>
       <c r="E51" t="s">
-        <v>172</v>
-      </c>
-      <c r="F51" t="s">
-        <v>149</v>
-      </c>
-      <c r="G51" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A52" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C52" t="s">
+        <v>166</v>
+      </c>
+      <c r="D52" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A53" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C53" t="s">
+        <v>166</v>
+      </c>
+      <c r="D53" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A54" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C54" t="s">
+        <v>166</v>
+      </c>
+      <c r="D54" t="s">
+        <v>27</v>
+      </c>
+      <c r="E54" t="s">
+        <v>153</v>
+      </c>
+      <c r="F54" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A55" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C55" t="s">
+        <v>166</v>
+      </c>
+      <c r="D55" t="s">
+        <v>315</v>
+      </c>
+      <c r="E55" t="s">
+        <v>153</v>
+      </c>
+      <c r="F55" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+      <c r="A56" s="3" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="52" spans="1:7" ht="174" x14ac:dyDescent="0.35">
-      <c r="A52" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="B52" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="C52" t="s">
-        <v>21</v>
-      </c>
-      <c r="D52" t="s">
-        <v>24</v>
-      </c>
-      <c r="E52" t="s">
-        <v>172</v>
-      </c>
-      <c r="F52" t="s">
-        <v>149</v>
-      </c>
-      <c r="G52" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="174" x14ac:dyDescent="0.35">
-      <c r="A53" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="C53" t="s">
-        <v>21</v>
-      </c>
-      <c r="D53" t="s">
-        <v>25</v>
-      </c>
-      <c r="E53" t="s">
-        <v>172</v>
-      </c>
-      <c r="F53" t="s">
-        <v>149</v>
-      </c>
-      <c r="G53" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="174" x14ac:dyDescent="0.35">
-      <c r="A54" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="C54" t="s">
-        <v>21</v>
-      </c>
-      <c r="D54" t="s">
-        <v>26</v>
-      </c>
-      <c r="E54" t="s">
-        <v>172</v>
-      </c>
-      <c r="F54" t="s">
-        <v>149</v>
-      </c>
-      <c r="G54" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" ht="174" x14ac:dyDescent="0.35">
-      <c r="A55" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="C55" t="s">
-        <v>21</v>
-      </c>
-      <c r="D55" t="s">
-        <v>27</v>
-      </c>
-      <c r="E55" t="s">
-        <v>172</v>
-      </c>
-      <c r="F55" t="s">
-        <v>149</v>
-      </c>
-      <c r="G55" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="174" x14ac:dyDescent="0.35">
-      <c r="A56" s="3" t="s">
-        <v>201</v>
-      </c>
       <c r="B56" s="3" t="s">
-        <v>239</v>
+        <v>167</v>
       </c>
       <c r="C56" t="s">
-        <v>21</v>
+        <v>166</v>
       </c>
       <c r="D56" t="s">
-        <v>28</v>
+        <v>134</v>
       </c>
       <c r="E56" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="F56" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="G56" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A57" s="3" t="s">
-        <v>202</v>
+        <v>170</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>204</v>
+        <v>290</v>
       </c>
       <c r="C57" t="s">
-        <v>21</v>
+        <v>166</v>
       </c>
       <c r="D57" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="E57" t="s">
-        <v>172</v>
-      </c>
-      <c r="F57" t="s">
-        <v>149</v>
-      </c>
-      <c r="G57" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A58" s="3" t="s">
-        <v>203</v>
+        <v>36</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>205</v>
+        <v>173</v>
       </c>
       <c r="C58" t="s">
-        <v>21</v>
+        <v>166</v>
       </c>
       <c r="D58" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E58" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="F58" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="G58" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="116" x14ac:dyDescent="0.35">
       <c r="A59" s="3" t="s">
-        <v>192</v>
+        <v>175</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>220</v>
+        <v>174</v>
       </c>
       <c r="C59" t="s">
         <v>21</v>
       </c>
       <c r="D59" t="s">
-        <v>32</v>
-      </c>
-      <c r="E59" t="s">
-        <v>172</v>
+        <v>38</v>
       </c>
       <c r="F59" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="G59" t="s">
-        <v>150</v>
+        <v>38</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A60" s="3" t="s">
-        <v>31</v>
+        <v>177</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>221</v>
+        <v>176</v>
       </c>
       <c r="C60" t="s">
         <v>21</v>
       </c>
       <c r="D60" t="s">
-        <v>33</v>
-      </c>
-      <c r="E60" t="s">
-        <v>172</v>
-      </c>
-      <c r="F60" t="s">
-        <v>149</v>
-      </c>
-      <c r="G60" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A61" s="3" t="s">
-        <v>110</v>
+        <v>178</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>222</v>
+        <v>179</v>
       </c>
       <c r="C61" t="s">
         <v>21</v>
       </c>
       <c r="D61" t="s">
-        <v>111</v>
-      </c>
-      <c r="E61" t="s">
-        <v>172</v>
+        <v>22</v>
       </c>
       <c r="F61" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="G61" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A62" s="3" t="s">
-        <v>116</v>
+        <v>186</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>224</v>
+        <v>185</v>
       </c>
       <c r="C62" t="s">
         <v>21</v>
       </c>
       <c r="D62" t="s">
-        <v>120</v>
+        <v>23</v>
       </c>
       <c r="E62" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="F62" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="G62" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A63" s="3" t="s">
-        <v>112</v>
+        <v>188</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>223</v>
+        <v>187</v>
       </c>
       <c r="C63" t="s">
         <v>21</v>
       </c>
       <c r="D63" t="s">
-        <v>113</v>
+        <v>24</v>
       </c>
       <c r="E63" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="F63" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="G63" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A64" s="3" t="s">
-        <v>117</v>
+        <v>171</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>224</v>
+        <v>189</v>
       </c>
       <c r="C64" t="s">
         <v>21</v>
       </c>
       <c r="D64" t="s">
-        <v>119</v>
+        <v>25</v>
       </c>
       <c r="E64" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="F64" t="s">
-        <v>149</v>
+        <v>131</v>
       </c>
       <c r="G64" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A65" s="3" t="s">
-        <v>121</v>
+        <v>191</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>225</v>
+        <v>190</v>
       </c>
       <c r="C65" t="s">
         <v>21</v>
       </c>
       <c r="D65" t="s">
-        <v>122</v>
+        <v>26</v>
       </c>
       <c r="E65" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+        <v>153</v>
+      </c>
+      <c r="F65" t="s">
+        <v>131</v>
+      </c>
+      <c r="G65" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A66" s="3" t="s">
-        <v>125</v>
+        <v>192</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>226</v>
+        <v>197</v>
       </c>
       <c r="C66" t="s">
         <v>21</v>
       </c>
       <c r="D66" t="s">
-        <v>123</v>
+        <v>27</v>
       </c>
       <c r="E66" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+        <v>153</v>
+      </c>
+      <c r="F66" t="s">
+        <v>131</v>
+      </c>
+      <c r="G66" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A67" s="3" t="s">
-        <v>126</v>
+        <v>180</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="C67" t="s">
         <v>21</v>
       </c>
       <c r="D67" t="s">
-        <v>124</v>
+        <v>28</v>
       </c>
       <c r="E67" t="s">
-        <v>172</v>
+        <v>153</v>
+      </c>
+      <c r="F67" t="s">
+        <v>131</v>
+      </c>
+      <c r="G67" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
-        <v>240</v>
+        <v>181</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>241</v>
+        <v>183</v>
       </c>
       <c r="C68" t="s">
         <v>21</v>
       </c>
       <c r="D68" t="s">
-        <v>152</v>
+        <v>29</v>
       </c>
       <c r="E68" t="s">
-        <v>172</v>
+        <v>153</v>
       </c>
       <c r="F68" t="s">
-        <v>153</v>
+        <v>131</v>
       </c>
       <c r="G68" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" ht="203" x14ac:dyDescent="0.35">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="174" x14ac:dyDescent="0.35">
       <c r="A69" s="3" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>237</v>
+        <v>184</v>
       </c>
       <c r="C69" t="s">
         <v>21</v>
       </c>
       <c r="D69" t="s">
-        <v>238</v>
+        <v>30</v>
       </c>
       <c r="E69" t="s">
+        <v>153</v>
+      </c>
+      <c r="F69" t="s">
+        <v>131</v>
+      </c>
+      <c r="G69" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+      <c r="A70" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="F69" t="s">
-        <v>171</v>
-      </c>
-      <c r="G69" t="s">
+      <c r="B70" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C70" t="s">
+        <v>21</v>
+      </c>
+      <c r="D70" t="s">
+        <v>32</v>
+      </c>
+      <c r="E70" t="s">
+        <v>153</v>
+      </c>
+      <c r="F70" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B70" s="3"/>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="B71" s="3"/>
+      <c r="G70" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+      <c r="A71" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="C71" t="s">
+        <v>21</v>
+      </c>
+      <c r="D71" t="s">
+        <v>33</v>
+      </c>
+      <c r="E71" t="s">
+        <v>153</v>
+      </c>
+      <c r="F71" t="s">
+        <v>131</v>
+      </c>
+      <c r="G71" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
+      <c r="A72" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C72" t="s">
+        <v>21</v>
+      </c>
+      <c r="D72" t="s">
+        <v>93</v>
+      </c>
+      <c r="E72" t="s">
+        <v>153</v>
+      </c>
+      <c r="F72" t="s">
+        <v>131</v>
+      </c>
+      <c r="G72" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A73" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C73" t="s">
+        <v>21</v>
+      </c>
+      <c r="D73" t="s">
+        <v>102</v>
+      </c>
+      <c r="E73" t="s">
+        <v>153</v>
+      </c>
+      <c r="F73" t="s">
+        <v>131</v>
+      </c>
+      <c r="G73" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" ht="304.5" x14ac:dyDescent="0.35">
+      <c r="A74" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="C74" t="s">
+        <v>21</v>
+      </c>
+      <c r="D74" t="s">
+        <v>95</v>
+      </c>
+      <c r="E74" t="s">
+        <v>153</v>
+      </c>
+      <c r="F74" t="s">
+        <v>131</v>
+      </c>
+      <c r="G74" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A75" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B75" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C75" t="s">
+        <v>21</v>
+      </c>
+      <c r="D75" t="s">
+        <v>101</v>
+      </c>
+      <c r="E75" t="s">
+        <v>153</v>
+      </c>
+      <c r="F75" t="s">
+        <v>131</v>
+      </c>
+      <c r="G75" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A76" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="C76" t="s">
+        <v>21</v>
+      </c>
+      <c r="D76" t="s">
+        <v>104</v>
+      </c>
+      <c r="E76" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A77" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C77" t="s">
+        <v>21</v>
+      </c>
+      <c r="D77" t="s">
+        <v>105</v>
+      </c>
+      <c r="E77" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="A78" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B78" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C78" t="s">
+        <v>21</v>
+      </c>
+      <c r="D78" t="s">
+        <v>106</v>
+      </c>
+      <c r="E78" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="174" x14ac:dyDescent="0.35">
+      <c r="A79" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C79" t="s">
+        <v>21</v>
+      </c>
+      <c r="D79" t="s">
+        <v>134</v>
+      </c>
+      <c r="E79" t="s">
+        <v>153</v>
+      </c>
+      <c r="F79" t="s">
+        <v>135</v>
+      </c>
+      <c r="G79" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" ht="203" x14ac:dyDescent="0.35">
+      <c r="A80" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B80" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="C80" t="s">
+        <v>21</v>
+      </c>
+      <c r="D80" t="s">
+        <v>216</v>
+      </c>
+      <c r="E80" t="s">
+        <v>153</v>
+      </c>
+      <c r="F80" t="s">
+        <v>152</v>
+      </c>
+      <c r="G80" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A81" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B81" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="C81" t="s">
+        <v>300</v>
+      </c>
+      <c r="D81" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A82" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C82" t="s">
+        <v>300</v>
+      </c>
+      <c r="D82" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A83" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="B83" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="C83" t="s">
+        <v>300</v>
+      </c>
+      <c r="D83" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A84" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="C84" t="s">
+        <v>300</v>
+      </c>
+      <c r="D84" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="58" x14ac:dyDescent="0.35">
+      <c r="A85" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="B85" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="C85" t="s">
+        <v>300</v>
+      </c>
+      <c r="D85" t="s">
+        <v>19</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B25" r:id="rId1" display="study.versions.studyDesigns.objectives@$ob.$ob.endpoints[level.code=&quot;C94496&quot;].{$ob.id: &quot;primary&quot;}" xr:uid="{74E81704-A140-48FF-9D58-8B18F3C8EA13}"/>
-    <hyperlink ref="B11" r:id="rId2" xr:uid="{546F8543-000B-4AD4-8472-81E6831062E9}"/>
+    <hyperlink ref="B12" r:id="rId1" xr:uid="{546F8543-000B-4AD4-8472-81E6831062E9}"/>
+    <hyperlink ref="B34" r:id="rId2" display="study.versions.studyDesigns.objectives@$ob.$ob.endpoints[level.code=&quot;C94496&quot;].{$ob.id: &quot;primary&quot;}" xr:uid="{74E81704-A140-48FF-9D58-8B18F3C8EA13}"/>
+    <hyperlink ref="B33" r:id="rId3" xr:uid="{99798F78-4BAF-4D31-B44E-B30A0F19703D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2995,7 +3528,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FC83523-A55B-4B95-86A9-D032F62CA141}">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.6328125" customWidth="1"/>
@@ -3004,17 +3537,17 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>179</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="3" customFormat="1" ht="45.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="B3" s="8"/>
     </row>
@@ -3022,7 +3555,7 @@
     <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -3030,7 +3563,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="29" x14ac:dyDescent="0.35">
@@ -3038,15 +3571,15 @@
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -3054,192 +3587,225 @@
         <v>2</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>175</v>
+        <v>287</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
-        <v>68</v>
+        <v>279</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="58" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>115</v>
+        <v>156</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" s="1" t="s">
+        <v>96</v>
+      </c>
       <c r="B28" s="3" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="58" x14ac:dyDescent="0.35">
+      <c r="B31" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>145</v>
+      </c>
       <c r="B34" s="3" t="s">
-        <v>155</v>
+        <v>257</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
-        <v>162</v>
+        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
-        <v>160</v>
+        <v>141</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" s="1" t="s">
-        <v>74</v>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="B44" s="3" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B46" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A48" s="1" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="49" spans="2:2" ht="29" x14ac:dyDescent="0.35">
-      <c r="B49" s="3" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B47" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="B48" s="3" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" s="1" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B51" s="6" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="52" spans="2:2" ht="29" x14ac:dyDescent="0.35">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B51" s="3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B52" s="6" t="s">
-        <v>218</v>
+        <v>195</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="29" x14ac:dyDescent="0.35">
+      <c r="B53" s="6" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B56" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B57" s="3" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B58" s="3" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -3252,15 +3818,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4">
@@ -3271,7 +3828,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100527ED9A1E2F34D48AA5925CCBA0CEC41" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="73c2da0cd5c8d9fd369ff3018c825410">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4" xmlns:ns3="985d26ac-cf7b-4687-94e0-26b141782da7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b3600b0f37fd05e6cabe55b41d10e7dc" ns2:_="" ns3:_="">
     <xsd:import namespace="c40ffa35-e506-4eb9-af8f-b5d6f9d0d5e4"/>
@@ -3466,15 +4023,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12DB76A7-ED98-4EE3-9432-17F601352CF4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E61FE636-68A4-4725-8134-F4B9672BB2E7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
@@ -3491,7 +4049,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9675DCA-D684-4E4E-B61D-0AB2D6821582}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3508,4 +4066,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12DB76A7-ED98-4EE3-9432-17F601352CF4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>